<commit_message>
generated new IOS bar graph (new order)
</commit_message>
<xml_diff>
--- a/SFN/Trust Behavioral Analysis/IOS/IOS.xlsx
+++ b/SFN/Trust Behavioral Analysis/IOS/IOS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/avidachs/Documents/GitHub/rf1-sra-trust/SFN/Trust Behavioral Analysis/IOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD064488-8BFC-1C4A-8CAE-CBA17B9626AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7978925A-02AD-6445-8384-5E0556994E5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{B1AA9258-5751-4D49-84BF-3D4F0F6CB9F5}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16120" xr2:uid="{B1AA9258-5751-4D49-84BF-3D4F0F6CB9F5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -51,12 +51,6 @@
     <t>NaN</t>
   </si>
   <si>
-    <t>Friend</t>
-  </si>
-  <si>
-    <t>Stranger</t>
-  </si>
-  <si>
     <t>Computer</t>
   </si>
   <si>
@@ -67,6 +61,12 @@
   </si>
   <si>
     <t>y</t>
+  </si>
+  <si>
+    <t>aFriend</t>
+  </si>
+  <si>
+    <t>bStranger</t>
   </si>
 </sst>
 </file>
@@ -423,18 +423,18 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B2">
         <v>5.0869565217391308</v>
@@ -445,7 +445,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B3">
         <v>1.8115942028985508</v>
@@ -456,7 +456,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B4">
         <v>1.8115942028985508</v>

</xml_diff>